<commit_message>
BOM: team spreadsheet updated (2026-09-21) — printed parts and all nine fastener lines now priced; stale 'unpriced' prose removed; McMaster-Carr vendor name; openpyxl pinned
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reference/bom/Duke_Humanoid_V2_BOM_WIP.xlsx
+++ b/reference/bom/Duke_Humanoid_V2_BOM_WIP.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="246">
   <si>
     <t>Category</t>
   </si>
@@ -490,7 +490,7 @@
     <t>P11</t>
   </si>
   <si>
-    <t>Gipper Rack, PLA</t>
+    <t>Gripper Rack, PLA</t>
   </si>
   <si>
     <t>P12</t>
@@ -670,28 +670,43 @@
     <t>45x58x7 Ball Bearing</t>
   </si>
   <si>
+    <t>https://www.amazon.com/XIKE-6809-2RS-Bearings-45x58x7mm-Pre-Lubricated/dp/B09D2J9P82</t>
+  </si>
+  <si>
     <t>H1</t>
   </si>
   <si>
     <t>50x65x7 Ball Bearing</t>
   </si>
   <si>
+    <t>https://www.amazon.com/uxcell-6810-2RS-Groove-Bearings-Double/dp/B082PYMQFL</t>
+  </si>
+  <si>
     <t>H2</t>
   </si>
   <si>
     <t>35x44x5 Ball Bearing</t>
   </si>
   <si>
+    <t>https://www.amazon.com/XIKE-6707-2RS-Bearings-35x44x5mm-Pre-Lubricated/dp/B09D2XN464/</t>
+  </si>
+  <si>
     <t>H3</t>
   </si>
   <si>
-    <t>35x47x7 Ball Bearing</t>
+    <t>35x47x7 6807-2RS Ball Bearing</t>
+  </si>
+  <si>
+    <t>https://www.amazon.com/XIKE-6807-2RS-Bearings-35x47x7mm-Pre-Lubricated/dp/B09D2ZHNPH/</t>
   </si>
   <si>
     <t>H4</t>
   </si>
   <si>
-    <t>30x37x4 Ball Bearing</t>
+    <t>30x37x4  6706-2RS Ball Bearing</t>
+  </si>
+  <si>
+    <t>https://www.amazon.com/XIKE-6706-2RS-Bearings-30x37x4mm-Pre-Lubricated/dp/B09D35XB19</t>
   </si>
   <si>
     <t>H5</t>
@@ -700,22 +715,34 @@
     <t>10x15x4 Ball Bearing</t>
   </si>
   <si>
+    <t>https://www.amazon.com/uxcell-6700-2RS-Groove-Bearings-Double/dp/B082PR3DFZ</t>
+  </si>
+  <si>
     <t>H6</t>
   </si>
   <si>
     <t>M3x10 Torx Button Head Screw</t>
   </si>
   <si>
+    <t>https://www.mcmaster.com/90991A114/</t>
+  </si>
+  <si>
     <t>H7</t>
   </si>
   <si>
     <t>M4x8 Torx Button Head Screw</t>
   </si>
   <si>
+    <t>https://www.mcmaster.com/90991A121/</t>
+  </si>
+  <si>
     <t>H8</t>
   </si>
   <si>
     <t>M4x10 Torx Button Head Screw</t>
+  </si>
+  <si>
+    <t>https://www.mcmaster.com/90942A118/</t>
   </si>
   <si>
     <t>Calibration</t>
@@ -732,7 +759,7 @@
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="$#,##0.00"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -798,6 +825,12 @@
       <u/>
       <color rgb="FF1155CC"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11.0"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="7">
@@ -927,14 +960,14 @@
     <xf borderId="0" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
+    <xf borderId="0" fillId="5" fontId="14" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
     <xf borderId="0" fillId="5" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="5" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="5" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="6" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
@@ -2801,21 +2834,24 @@
       <c r="D63" s="22"/>
       <c r="E63" s="23">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.9560332502</v>
       </c>
       <c r="F63" s="22">
         <v>2.0</v>
       </c>
       <c r="G63" s="24">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1.9120665</v>
+      </c>
+      <c r="I63" s="3">
+        <v>0.07666666</v>
       </c>
       <c r="J63" s="3">
         <v>12.47</v>
       </c>
       <c r="K63" s="25">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>0.9560332502</v>
       </c>
     </row>
     <row r="64">
@@ -2831,21 +2867,24 @@
       <c r="D64" s="22"/>
       <c r="E64" s="23">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.55934185</v>
       </c>
       <c r="F64" s="22">
         <v>4.0</v>
       </c>
       <c r="G64" s="24">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>2.2373674</v>
+      </c>
+      <c r="I64" s="3">
+        <v>0.044855</v>
       </c>
       <c r="J64" s="3">
         <v>12.47</v>
       </c>
       <c r="K64" s="25">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>0.55934185</v>
       </c>
     </row>
     <row r="65">
@@ -2861,21 +2900,24 @@
       <c r="D65" s="22"/>
       <c r="E65" s="23">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.128871</v>
       </c>
       <c r="F65" s="22">
         <v>2.0</v>
       </c>
       <c r="G65" s="24">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.257742</v>
+      </c>
+      <c r="I65" s="3">
+        <v>0.00129</v>
       </c>
       <c r="J65" s="3">
         <v>99.9</v>
       </c>
       <c r="K65" s="25">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>0.128871</v>
       </c>
     </row>
     <row r="66">
@@ -2891,21 +2933,24 @@
       <c r="D66" s="22"/>
       <c r="E66" s="23">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.4233565</v>
       </c>
       <c r="F66" s="22">
         <v>4.0</v>
       </c>
       <c r="G66" s="24">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1.693426</v>
+      </c>
+      <c r="I66" s="3">
+        <v>0.03395</v>
       </c>
       <c r="J66" s="3">
         <v>12.47</v>
       </c>
       <c r="K66" s="25">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>0.4233565</v>
       </c>
     </row>
     <row r="67">
@@ -2921,21 +2966,24 @@
       <c r="D67" s="22"/>
       <c r="E67" s="23">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.04070208</v>
       </c>
       <c r="F67" s="22">
         <v>4.0</v>
       </c>
       <c r="G67" s="24">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.16280832</v>
+      </c>
+      <c r="I67" s="3">
+        <v>0.003264</v>
       </c>
       <c r="J67" s="3">
         <v>12.47</v>
       </c>
       <c r="K67" s="25">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>0.04070208</v>
       </c>
     </row>
     <row r="68">
@@ -2951,21 +2999,24 @@
       <c r="D68" s="22"/>
       <c r="E68" s="23">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.017458</v>
       </c>
       <c r="F68" s="22">
         <v>12.0</v>
       </c>
       <c r="G68" s="24">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.209496</v>
+      </c>
+      <c r="I68" s="3">
+        <v>0.0014</v>
       </c>
       <c r="J68" s="3">
         <v>12.47</v>
       </c>
       <c r="K68" s="25">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>0.017458</v>
       </c>
     </row>
     <row r="69">
@@ -2981,21 +3032,24 @@
       <c r="D69" s="22"/>
       <c r="E69" s="23">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.6481906</v>
       </c>
       <c r="F69" s="22">
         <v>2.0</v>
       </c>
       <c r="G69" s="24">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1.2963812</v>
+      </c>
+      <c r="I69" s="3">
+        <v>0.05198</v>
       </c>
       <c r="J69" s="3">
         <v>12.47</v>
       </c>
       <c r="K69" s="25">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>0.6481906</v>
       </c>
     </row>
     <row r="70">
@@ -3011,21 +3065,24 @@
       <c r="D70" s="22"/>
       <c r="E70" s="23">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.46940821</v>
       </c>
       <c r="F70" s="22">
         <v>2.0</v>
       </c>
       <c r="G70" s="24">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.93881642</v>
+      </c>
+      <c r="I70" s="3">
+        <v>0.037643</v>
       </c>
       <c r="J70" s="3">
         <v>12.47</v>
       </c>
       <c r="K70" s="25">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>0.46940821</v>
       </c>
     </row>
     <row r="71">
@@ -3041,21 +3098,24 @@
       <c r="D71" s="22"/>
       <c r="E71" s="23">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.15556325</v>
       </c>
       <c r="F71" s="22">
         <v>2.0</v>
       </c>
       <c r="G71" s="24">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.3111265</v>
+      </c>
+      <c r="I71" s="3">
+        <v>0.012475</v>
       </c>
       <c r="J71" s="3">
         <v>12.47</v>
       </c>
       <c r="K71" s="25">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>0.15556325</v>
       </c>
     </row>
     <row r="72">
@@ -3071,21 +3131,24 @@
       <c r="D72" s="22"/>
       <c r="E72" s="23">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.15092441</v>
       </c>
       <c r="F72" s="22">
         <v>2.0</v>
       </c>
       <c r="G72" s="24">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.30184882</v>
+      </c>
+      <c r="I72" s="3">
+        <v>0.012103</v>
       </c>
       <c r="J72" s="3">
         <v>12.47</v>
       </c>
       <c r="K72" s="25">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>0.15092441</v>
       </c>
     </row>
     <row r="73">
@@ -3101,21 +3164,24 @@
       <c r="D73" s="22"/>
       <c r="E73" s="23">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1.08797906</v>
       </c>
       <c r="F73" s="22">
         <v>2.0</v>
       </c>
       <c r="G73" s="24">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>2.17595812</v>
+      </c>
+      <c r="I73" s="3">
+        <v>0.031094</v>
       </c>
       <c r="J73" s="3">
         <v>34.99</v>
       </c>
       <c r="K73" s="25">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>1.08797906</v>
       </c>
     </row>
     <row r="74">
@@ -3131,21 +3197,24 @@
       <c r="D74" s="22"/>
       <c r="E74" s="23">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1.08797906</v>
       </c>
       <c r="F74" s="22">
         <v>2.0</v>
       </c>
       <c r="G74" s="24">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>2.17595812</v>
+      </c>
+      <c r="I74" s="3">
+        <v>0.031094</v>
       </c>
       <c r="J74" s="3">
         <v>34.99</v>
       </c>
       <c r="K74" s="25">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>1.08797906</v>
       </c>
     </row>
     <row r="75">
@@ -3161,21 +3230,24 @@
       <c r="D75" s="22"/>
       <c r="E75" s="23">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.90841038</v>
       </c>
       <c r="F75" s="22">
         <v>2.0</v>
       </c>
       <c r="G75" s="24">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1.81682076</v>
+      </c>
+      <c r="I75" s="3">
+        <v>0.025962</v>
       </c>
       <c r="J75" s="3">
         <v>34.99</v>
       </c>
       <c r="K75" s="25">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>0.90841038</v>
       </c>
     </row>
     <row r="76">
@@ -3191,21 +3263,24 @@
       <c r="D76" s="22"/>
       <c r="E76" s="23">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.90841038</v>
       </c>
       <c r="F76" s="22">
         <v>2.0</v>
       </c>
       <c r="G76" s="24">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1.81682076</v>
+      </c>
+      <c r="I76" s="3">
+        <v>0.025962</v>
       </c>
       <c r="J76" s="3">
         <v>34.99</v>
       </c>
       <c r="K76" s="25">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>0.90841038</v>
       </c>
     </row>
     <row r="77">
@@ -3221,21 +3296,24 @@
       <c r="D77" s="22"/>
       <c r="E77" s="23">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1.08797906</v>
       </c>
       <c r="F77" s="22">
         <v>2.0</v>
       </c>
       <c r="G77" s="24">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>2.17595812</v>
+      </c>
+      <c r="I77" s="3">
+        <v>0.031094</v>
       </c>
       <c r="J77" s="3">
         <v>34.99</v>
       </c>
       <c r="K77" s="25">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>1.08797906</v>
       </c>
     </row>
     <row r="78">
@@ -3251,21 +3329,24 @@
       <c r="D78" s="22"/>
       <c r="E78" s="23">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1.08797906</v>
       </c>
       <c r="F78" s="22">
         <v>2.0</v>
       </c>
       <c r="G78" s="24">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>2.17595812</v>
+      </c>
+      <c r="I78" s="3">
+        <v>0.031094</v>
       </c>
       <c r="J78" s="3">
         <v>34.99</v>
       </c>
       <c r="K78" s="25">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>1.08797906</v>
       </c>
     </row>
     <row r="79">
@@ -3281,21 +3362,24 @@
       <c r="D79" s="22"/>
       <c r="E79" s="23">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.91530341</v>
       </c>
       <c r="F79" s="22">
         <v>2.0</v>
       </c>
       <c r="G79" s="24">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1.83060682</v>
+      </c>
+      <c r="I79" s="3">
+        <v>0.026159</v>
       </c>
       <c r="J79" s="3">
         <v>34.99</v>
       </c>
       <c r="K79" s="25">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>0.91530341</v>
       </c>
     </row>
     <row r="80">
@@ -3311,21 +3395,24 @@
       <c r="D80" s="22"/>
       <c r="E80" s="23">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.91530341</v>
       </c>
       <c r="F80" s="22">
         <v>2.0</v>
       </c>
       <c r="G80" s="24">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1.83060682</v>
+      </c>
+      <c r="I80" s="3">
+        <v>0.026159</v>
       </c>
       <c r="J80" s="3">
         <v>34.99</v>
       </c>
       <c r="K80" s="25">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>0.91530341</v>
       </c>
     </row>
     <row r="81">
@@ -3341,21 +3428,24 @@
       <c r="D81" s="22"/>
       <c r="E81" s="23">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1.56454286</v>
       </c>
       <c r="F81" s="22">
         <v>4.0</v>
       </c>
       <c r="G81" s="24">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>6.25817144</v>
+      </c>
+      <c r="I81" s="3">
+        <v>0.044714</v>
       </c>
       <c r="J81" s="3">
         <v>34.99</v>
       </c>
       <c r="K81" s="25">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>1.56454286</v>
       </c>
     </row>
     <row r="82">
@@ -3371,21 +3461,24 @@
       <c r="D82" s="22"/>
       <c r="E82" s="23">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.58401809</v>
       </c>
       <c r="F82" s="22">
         <v>2.0</v>
       </c>
       <c r="G82" s="24">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1.16803618</v>
+      </c>
+      <c r="I82" s="3">
+        <v>0.016691</v>
       </c>
       <c r="J82" s="3">
         <v>34.99</v>
       </c>
       <c r="K82" s="25">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>0.58401809</v>
       </c>
     </row>
     <row r="83">
@@ -3401,21 +3494,24 @@
       <c r="D83" s="22"/>
       <c r="E83" s="23">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.58401809</v>
       </c>
       <c r="F83" s="22">
         <v>2.0</v>
       </c>
       <c r="G83" s="24">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1.16803618</v>
+      </c>
+      <c r="I83" s="3">
+        <v>0.016691</v>
       </c>
       <c r="J83" s="3">
         <v>34.99</v>
       </c>
       <c r="K83" s="25">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>0.58401809</v>
       </c>
     </row>
     <row r="84">
@@ -3431,21 +3527,24 @@
       <c r="D84" s="22"/>
       <c r="E84" s="23">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.48622104</v>
       </c>
       <c r="F84" s="22">
         <v>2.0</v>
       </c>
       <c r="G84" s="24">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.97244208</v>
+      </c>
+      <c r="I84" s="3">
+        <v>0.013896</v>
       </c>
       <c r="J84" s="3">
         <v>34.99</v>
       </c>
       <c r="K84" s="25">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>0.48622104</v>
       </c>
     </row>
     <row r="85">
@@ -3461,21 +3560,24 @@
       <c r="D85" s="22"/>
       <c r="E85" s="23">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>4.14155636</v>
       </c>
       <c r="F85" s="22">
         <v>2.0</v>
       </c>
       <c r="G85" s="24">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>8.28311272</v>
+      </c>
+      <c r="I85" s="3">
+        <v>0.118364</v>
       </c>
       <c r="J85" s="3">
         <v>34.99</v>
       </c>
       <c r="K85" s="25">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>4.14155636</v>
       </c>
     </row>
     <row r="86">
@@ -3491,21 +3593,24 @@
       <c r="D86" s="22"/>
       <c r="E86" s="23">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.43576546</v>
       </c>
       <c r="F86" s="22">
         <v>2.0</v>
       </c>
       <c r="G86" s="24">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.87153092</v>
+      </c>
+      <c r="I86" s="3">
+        <v>0.012454</v>
       </c>
       <c r="J86" s="3">
         <v>34.99</v>
       </c>
       <c r="K86" s="25">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>0.43576546</v>
       </c>
     </row>
     <row r="87">
@@ -3521,21 +3626,24 @@
       <c r="D87" s="22"/>
       <c r="E87" s="23">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.43576546</v>
       </c>
       <c r="F87" s="22">
         <v>2.0</v>
       </c>
       <c r="G87" s="24">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.87153092</v>
+      </c>
+      <c r="I87" s="3">
+        <v>0.012454</v>
       </c>
       <c r="J87" s="3">
         <v>34.99</v>
       </c>
       <c r="K87" s="25">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>0.43576546</v>
       </c>
     </row>
     <row r="88">
@@ -3551,21 +3659,24 @@
       <c r="D88" s="22"/>
       <c r="E88" s="23">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.29087187</v>
       </c>
       <c r="F88" s="22">
         <v>4.0</v>
       </c>
       <c r="G88" s="24">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1.16348748</v>
+      </c>
+      <c r="I88" s="3">
+        <v>0.008313</v>
       </c>
       <c r="J88" s="3">
         <v>34.99</v>
       </c>
       <c r="K88" s="25">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>0.29087187</v>
       </c>
     </row>
     <row r="89">
@@ -3581,21 +3692,24 @@
       <c r="D89" s="22"/>
       <c r="E89" s="23">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.29087187</v>
       </c>
       <c r="F89" s="22">
         <v>4.0</v>
       </c>
       <c r="G89" s="24">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1.16348748</v>
+      </c>
+      <c r="I89" s="3">
+        <v>0.008313</v>
       </c>
       <c r="J89" s="3">
         <v>34.99</v>
       </c>
       <c r="K89" s="25">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>0.29087187</v>
       </c>
     </row>
     <row r="90">
@@ -3611,21 +3725,24 @@
       <c r="D90" s="22"/>
       <c r="E90" s="23">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.21427876</v>
       </c>
       <c r="F90" s="22">
         <v>2.0</v>
       </c>
       <c r="G90" s="24">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.42855752</v>
+      </c>
+      <c r="I90" s="3">
+        <v>0.006124</v>
       </c>
       <c r="J90" s="3">
         <v>34.99</v>
       </c>
       <c r="K90" s="25">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>0.21427876</v>
       </c>
     </row>
     <row r="91">
@@ -3641,21 +3758,24 @@
       <c r="D91" s="22"/>
       <c r="E91" s="23">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.21427876</v>
       </c>
       <c r="F91" s="22">
         <v>2.0</v>
       </c>
       <c r="G91" s="24">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.42855752</v>
+      </c>
+      <c r="I91" s="3">
+        <v>0.006124</v>
       </c>
       <c r="J91" s="3">
         <v>34.99</v>
       </c>
       <c r="K91" s="25">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>0.21427876</v>
       </c>
     </row>
     <row r="92">
@@ -3671,21 +3791,24 @@
       <c r="D92" s="22"/>
       <c r="E92" s="23">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>0.26672877</v>
       </c>
       <c r="F92" s="22">
         <v>8.0</v>
       </c>
       <c r="G92" s="24">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>2.13383016</v>
+      </c>
+      <c r="I92" s="3">
+        <v>0.007623</v>
       </c>
       <c r="J92" s="3">
         <v>34.99</v>
       </c>
       <c r="K92" s="25">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>0.26672877</v>
       </c>
     </row>
     <row r="93">
@@ -3698,14 +3821,18 @@
       <c r="C93" s="27" t="s">
         <v>218</v>
       </c>
-      <c r="D93" s="27"/>
-      <c r="E93" s="28"/>
+      <c r="D93" s="28" t="s">
+        <v>219</v>
+      </c>
+      <c r="E93" s="29">
+        <v>3.0</v>
+      </c>
       <c r="F93" s="27">
         <v>13.0</v>
       </c>
-      <c r="G93" s="29">
-        <f t="shared" si="2"/>
-        <v>0</v>
+      <c r="G93" s="30">
+        <f t="shared" si="2"/>
+        <v>39</v>
       </c>
     </row>
     <row r="94">
@@ -3713,19 +3840,23 @@
         <v>216</v>
       </c>
       <c r="B94" s="27" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C94" s="27" t="s">
-        <v>220</v>
-      </c>
-      <c r="D94" s="30"/>
-      <c r="E94" s="28"/>
+        <v>221</v>
+      </c>
+      <c r="D94" s="28" t="s">
+        <v>222</v>
+      </c>
+      <c r="E94" s="29">
+        <v>4.0</v>
+      </c>
       <c r="F94" s="27">
         <v>2.0</v>
       </c>
-      <c r="G94" s="29">
-        <f t="shared" si="2"/>
-        <v>0</v>
+      <c r="G94" s="30">
+        <f t="shared" si="2"/>
+        <v>8</v>
       </c>
     </row>
     <row r="95">
@@ -3733,19 +3864,23 @@
         <v>216</v>
       </c>
       <c r="B95" s="27" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="C95" s="27" t="s">
-        <v>222</v>
-      </c>
-      <c r="D95" s="30"/>
-      <c r="E95" s="28"/>
+        <v>224</v>
+      </c>
+      <c r="D95" s="28" t="s">
+        <v>225</v>
+      </c>
+      <c r="E95" s="29">
+        <v>3.0</v>
+      </c>
       <c r="F95" s="27">
         <v>18.0</v>
       </c>
-      <c r="G95" s="29">
-        <f t="shared" si="2"/>
-        <v>0</v>
+      <c r="G95" s="30">
+        <f t="shared" si="2"/>
+        <v>54</v>
       </c>
     </row>
     <row r="96">
@@ -3753,19 +3888,23 @@
         <v>216</v>
       </c>
       <c r="B96" s="27" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="C96" s="27" t="s">
-        <v>224</v>
-      </c>
-      <c r="D96" s="30"/>
-      <c r="E96" s="28"/>
+        <v>227</v>
+      </c>
+      <c r="D96" s="28" t="s">
+        <v>228</v>
+      </c>
+      <c r="E96" s="29">
+        <v>4.0</v>
+      </c>
       <c r="F96" s="27">
         <v>4.0</v>
       </c>
-      <c r="G96" s="29">
-        <f t="shared" si="2"/>
-        <v>0</v>
+      <c r="G96" s="30">
+        <f t="shared" si="2"/>
+        <v>16</v>
       </c>
     </row>
     <row r="97">
@@ -3773,19 +3912,23 @@
         <v>216</v>
       </c>
       <c r="B97" s="27" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="C97" s="27" t="s">
-        <v>226</v>
-      </c>
-      <c r="D97" s="30"/>
-      <c r="E97" s="28"/>
+        <v>230</v>
+      </c>
+      <c r="D97" s="28" t="s">
+        <v>231</v>
+      </c>
+      <c r="E97" s="29">
+        <v>2.0</v>
+      </c>
       <c r="F97" s="27">
         <v>2.0</v>
       </c>
-      <c r="G97" s="29">
-        <f t="shared" si="2"/>
-        <v>0</v>
+      <c r="G97" s="30">
+        <f t="shared" si="2"/>
+        <v>4</v>
       </c>
     </row>
     <row r="98">
@@ -3793,19 +3936,23 @@
         <v>216</v>
       </c>
       <c r="B98" s="27" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="C98" s="27" t="s">
-        <v>228</v>
-      </c>
-      <c r="D98" s="30"/>
-      <c r="E98" s="28"/>
+        <v>233</v>
+      </c>
+      <c r="D98" s="28" t="s">
+        <v>234</v>
+      </c>
+      <c r="E98" s="29">
+        <v>1.0</v>
+      </c>
       <c r="F98" s="27">
         <v>2.0</v>
       </c>
-      <c r="G98" s="29">
-        <f t="shared" si="2"/>
-        <v>0</v>
+      <c r="G98" s="30">
+        <f t="shared" si="2"/>
+        <v>2</v>
       </c>
     </row>
     <row r="99">
@@ -3813,17 +3960,23 @@
         <v>216</v>
       </c>
       <c r="B99" s="27" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
       <c r="C99" s="27" t="s">
-        <v>230</v>
-      </c>
-      <c r="D99" s="30"/>
-      <c r="E99" s="28"/>
-      <c r="F99" s="27"/>
-      <c r="G99" s="29">
-        <f t="shared" si="2"/>
-        <v>0</v>
+        <v>236</v>
+      </c>
+      <c r="D99" s="28" t="s">
+        <v>237</v>
+      </c>
+      <c r="E99" s="29">
+        <v>5.16</v>
+      </c>
+      <c r="F99" s="27">
+        <v>5.0</v>
+      </c>
+      <c r="G99" s="30">
+        <f t="shared" si="2"/>
+        <v>25.8</v>
       </c>
     </row>
     <row r="100">
@@ -3831,17 +3984,23 @@
         <v>216</v>
       </c>
       <c r="B100" s="27" t="s">
-        <v>231</v>
+        <v>238</v>
       </c>
       <c r="C100" s="27" t="s">
-        <v>232</v>
-      </c>
-      <c r="D100" s="30"/>
-      <c r="E100" s="28"/>
-      <c r="F100" s="27"/>
-      <c r="G100" s="29">
-        <f t="shared" si="2"/>
-        <v>0</v>
+        <v>239</v>
+      </c>
+      <c r="D100" s="28" t="s">
+        <v>240</v>
+      </c>
+      <c r="E100" s="29">
+        <v>7.2</v>
+      </c>
+      <c r="F100" s="27">
+        <v>1.0</v>
+      </c>
+      <c r="G100" s="30">
+        <f t="shared" si="2"/>
+        <v>7.2</v>
       </c>
     </row>
     <row r="101">
@@ -3849,22 +4008,28 @@
         <v>216</v>
       </c>
       <c r="B101" s="27" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
       <c r="C101" s="27" t="s">
-        <v>234</v>
-      </c>
-      <c r="D101" s="30"/>
-      <c r="E101" s="28"/>
-      <c r="F101" s="27"/>
-      <c r="G101" s="29">
-        <f t="shared" si="2"/>
-        <v>0</v>
+        <v>242</v>
+      </c>
+      <c r="D101" s="28" t="s">
+        <v>243</v>
+      </c>
+      <c r="E101" s="29">
+        <v>5.78</v>
+      </c>
+      <c r="F101" s="27">
+        <v>4.0</v>
+      </c>
+      <c r="G101" s="30">
+        <f t="shared" si="2"/>
+        <v>23.12</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="31" t="s">
-        <v>235</v>
+        <v>244</v>
       </c>
       <c r="B102" s="31"/>
       <c r="C102" s="32"/>
@@ -3887,19 +4052,19 @@
     </row>
     <row r="104">
       <c r="A104" s="3" t="s">
-        <v>236</v>
+        <v>245</v>
       </c>
       <c r="E104" s="35">
         <f>SUMPRODUCT(E2:E102, F2:F102)</f>
-        <v>12345.9485</v>
+        <v>12575.29904</v>
       </c>
       <c r="F104" s="25">
         <f t="shared" ref="F104:G104" si="5">SUM(F2:F102)</f>
-        <v>289</v>
+        <v>299</v>
       </c>
       <c r="G104" s="36">
         <f t="shared" si="5"/>
-        <v>12345.9485</v>
+        <v>12575.29904</v>
       </c>
     </row>
     <row r="105">
@@ -7742,7 +7907,16 @@
     <hyperlink r:id="rId40" ref="H21"/>
     <hyperlink r:id="rId41" ref="D22"/>
     <hyperlink r:id="rId42" ref="H22"/>
+    <hyperlink r:id="rId43" ref="D93"/>
+    <hyperlink r:id="rId44" ref="D94"/>
+    <hyperlink r:id="rId45" ref="D95"/>
+    <hyperlink r:id="rId46" ref="D96"/>
+    <hyperlink r:id="rId47" ref="D97"/>
+    <hyperlink r:id="rId48" ref="D98"/>
+    <hyperlink r:id="rId49" ref="D99"/>
+    <hyperlink r:id="rId50" ref="D100"/>
+    <hyperlink r:id="rId51" ref="D101"/>
   </hyperlinks>
-  <drawing r:id="rId43"/>
+  <drawing r:id="rId52"/>
 </worksheet>
 </file>
</xml_diff>